<commit_message>
Blank Commit cannot see what was changed. Seems to be an error?
</commit_message>
<xml_diff>
--- a/Installation_IDs.xlsx
+++ b/Installation_IDs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\RStor\CEMML\ClimateChange\Document Standards\Templates\TEMPLATES_SME_Word_Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3900F204-82F0-4007-B7F0-AB0ACFBA2B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8641C3E-162B-4A8B-A995-0130C21D96E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AIR FORCE" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="117">
   <si>
     <t>SITEID</t>
   </si>
@@ -335,13 +335,55 @@
   </si>
   <si>
     <t>Naval Submarine Base Kings Bay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joint Base Pearl Harbor-Hickam Sites - Main Base and Surrounding Areas (Zone 1) </t>
+  </si>
+  <si>
+    <t>Joint Base Pearl Harbor-Hickam Sites - Wahiawa Annex (Zone 3)</t>
+  </si>
+  <si>
+    <t>Joint Base Pearl Harbor-Hickam Sites - Lualualei Annex and Kalaeloa (Zone 2)</t>
+  </si>
+  <si>
+    <t>Naval Air Station Whidbey Island Sites</t>
+  </si>
+  <si>
+    <t>N62688</t>
+  </si>
+  <si>
+    <t>N32446-LF</t>
+  </si>
+  <si>
+    <t>N69212</t>
+  </si>
+  <si>
+    <t>Installation ID (Site Code)</t>
+  </si>
+  <si>
+    <t>N61008</t>
+  </si>
+  <si>
+    <t>N60201</t>
+  </si>
+  <si>
+    <t>N00207</t>
+  </si>
+  <si>
+    <t>N42237</t>
+  </si>
+  <si>
+    <t>N62813</t>
+  </si>
+  <si>
+    <t>N00620</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -366,13 +408,18 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -392,21 +439,27 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{0CA8EF0B-0BDB-4DAF-B59A-3C1C782D2818}"/>
+    <cellStyle name="Normal 3" xfId="2" xr:uid="{D3090902-139A-4C8F-A1F3-70510EFC808B}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -685,16 +738,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D94"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.6640625" customWidth="1"/>
-    <col min="2" max="2" width="67.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.33203125" customWidth="1"/>
+    <col min="1" max="1" width="7.7109375" customWidth="1"/>
+    <col min="2" max="2" width="67.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.28515625" customWidth="1"/>
     <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="6" max="6" width="24.44140625" customWidth="1"/>
+    <col min="6" max="6" width="24.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -704,7 +757,7 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -712,7 +765,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3</v>
       </c>
@@ -720,7 +773,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4</v>
       </c>
@@ -728,7 +781,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>5</v>
       </c>
@@ -736,7 +789,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>6</v>
       </c>
@@ -744,7 +797,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>7</v>
       </c>
@@ -752,7 +805,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>8</v>
       </c>
@@ -760,7 +813,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>9</v>
       </c>
@@ -768,7 +821,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>10</v>
       </c>
@@ -776,7 +829,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>11</v>
       </c>
@@ -784,7 +837,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>12</v>
       </c>
@@ -792,7 +845,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>13</v>
       </c>
@@ -800,7 +853,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>14</v>
       </c>
@@ -808,7 +861,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>15</v>
       </c>
@@ -816,7 +869,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>16</v>
       </c>
@@ -824,7 +877,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>17</v>
       </c>
@@ -832,7 +885,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>18</v>
       </c>
@@ -840,7 +893,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>19</v>
       </c>
@@ -848,7 +901,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>20</v>
       </c>
@@ -856,7 +909,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>21</v>
       </c>
@@ -864,7 +917,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>22</v>
       </c>
@@ -872,7 +925,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>23</v>
       </c>
@@ -880,7 +933,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>24</v>
       </c>
@@ -888,7 +941,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>25</v>
       </c>
@@ -896,7 +949,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>26</v>
       </c>
@@ -904,7 +957,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>27</v>
       </c>
@@ -912,7 +965,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>28</v>
       </c>
@@ -920,7 +973,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>29</v>
       </c>
@@ -928,7 +981,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>30</v>
       </c>
@@ -936,7 +989,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>31</v>
       </c>
@@ -944,7 +997,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>32</v>
       </c>
@@ -952,7 +1005,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>33</v>
       </c>
@@ -960,7 +1013,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>34</v>
       </c>
@@ -968,7 +1021,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>35</v>
       </c>
@@ -976,7 +1029,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>36</v>
       </c>
@@ -984,7 +1037,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>37</v>
       </c>
@@ -992,7 +1045,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>38</v>
       </c>
@@ -1000,7 +1053,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>39</v>
       </c>
@@ -1008,7 +1061,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>40</v>
       </c>
@@ -1016,7 +1069,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>41</v>
       </c>
@@ -1024,7 +1077,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>42</v>
       </c>
@@ -1032,7 +1085,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>43</v>
       </c>
@@ -1040,7 +1093,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>44</v>
       </c>
@@ -1048,7 +1101,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>45</v>
       </c>
@@ -1056,7 +1109,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>46</v>
       </c>
@@ -1064,7 +1117,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>47</v>
       </c>
@@ -1072,7 +1125,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>48</v>
       </c>
@@ -1080,7 +1133,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>49</v>
       </c>
@@ -1088,7 +1141,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>50</v>
       </c>
@@ -1096,7 +1149,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>51</v>
       </c>
@@ -1104,7 +1157,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>52</v>
       </c>
@@ -1112,7 +1165,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>53</v>
       </c>
@@ -1120,7 +1173,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>55</v>
       </c>
@@ -1128,7 +1181,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>56</v>
       </c>
@@ -1136,7 +1189,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>57</v>
       </c>
@@ -1144,7 +1197,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>58</v>
       </c>
@@ -1152,7 +1205,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>61</v>
       </c>
@@ -1160,7 +1213,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>62</v>
       </c>
@@ -1168,7 +1221,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>65</v>
       </c>
@@ -1176,7 +1229,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>66</v>
       </c>
@@ -1184,7 +1237,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>67</v>
       </c>
@@ -1192,7 +1245,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>69</v>
       </c>
@@ -1200,7 +1253,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>70</v>
       </c>
@@ -1208,7 +1261,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>71</v>
       </c>
@@ -1216,7 +1269,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>72</v>
       </c>
@@ -1224,7 +1277,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>73</v>
       </c>
@@ -1232,7 +1285,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>74</v>
       </c>
@@ -1240,7 +1293,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>75</v>
       </c>
@@ -1248,7 +1301,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>76</v>
       </c>
@@ -1256,7 +1309,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>77</v>
       </c>
@@ -1264,7 +1317,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>78</v>
       </c>
@@ -1272,7 +1325,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>79</v>
       </c>
@@ -1280,7 +1333,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>80</v>
       </c>
@@ -1288,7 +1341,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>81</v>
       </c>
@@ -1296,7 +1349,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>82</v>
       </c>
@@ -1304,7 +1357,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>83</v>
       </c>
@@ -1312,7 +1365,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>84</v>
       </c>
@@ -1320,7 +1373,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>85</v>
       </c>
@@ -1328,7 +1381,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>86</v>
       </c>
@@ -1336,7 +1389,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>87</v>
       </c>
@@ -1344,7 +1397,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>88</v>
       </c>
@@ -1352,7 +1405,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>89</v>
       </c>
@@ -1360,7 +1413,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>90</v>
       </c>
@@ -1368,7 +1421,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>91</v>
       </c>
@@ -1376,7 +1429,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>92</v>
       </c>
@@ -1384,7 +1437,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>93</v>
       </c>
@@ -1392,7 +1445,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>94</v>
       </c>
@@ -1400,7 +1453,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>95</v>
       </c>
@@ -1408,7 +1461,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>96</v>
       </c>
@@ -1416,7 +1469,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>97</v>
       </c>
@@ -1424,7 +1477,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>98</v>
       </c>
@@ -1432,7 +1485,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>99</v>
       </c>
@@ -1440,7 +1493,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>100</v>
       </c>
@@ -1455,78 +1508,145 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A06A16C-6F98-439D-96DD-17D8D49F3FE1}">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="41.109375" customWidth="1"/>
+    <col min="1" max="1" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="74.28515625" customWidth="1"/>
+    <col min="3" max="3" width="29" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C2" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C3" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5" s="6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C6" s="6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C7" s="6" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B9" s="3"/>
+      <c r="C8" s="6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>116</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>